<commit_message>
Update attendees-per-city average to 870, refresh source spreadsheet
Replaces assets/tour-2027-numbers.xlsx with the corrected file (its
own summary note now reads "92 cities" instead of "94", matching the
itinerary section already on the page).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/tour-2027-numbers.xlsx
+++ b/assets/tour-2027-numbers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/regulocastrogomez/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E2508DD-5E53-1A49-B157-906974A97B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650DCAA3-FACB-E049-B673-D2D627B5A89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16660" xr2:uid="{BBF3B1B2-2BD0-D242-B940-7BB9A5C7F668}"/>
   </bookViews>
@@ -347,7 +347,7 @@
     <t xml:space="preserve">*Note cost in USD </t>
   </si>
   <si>
-    <t>16 tours - 94 cities in total</t>
+    <t>16 tours - 92 cities in total</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Add August to the Tour 2027 Itinerary
The updated spreadsheet splits out a previously-unlabeled USA leg
(Houston, Dallas, San Antonio, Austin, Fort Worth, El Paso) as its own
August month, moving it out of July. Itinerary grid now covers all 12
months instead of 11; totals unchanged (92 cities, 80,350 attendees).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/tour-2027-numbers.xlsx
+++ b/assets/tour-2027-numbers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/regulocastrogomez/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650DCAA3-FACB-E049-B673-D2D627B5A89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86321418-ED0D-7648-A2A6-C757493927C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16660" xr2:uid="{BBF3B1B2-2BD0-D242-B940-7BB9A5C7F668}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="104">
   <si>
     <t>CD. JUAREZ</t>
   </si>
@@ -348,6 +348,9 @@
   </si>
   <si>
     <t>16 tours - 92 cities in total</t>
+  </si>
+  <si>
+    <t>AUGUST</t>
   </si>
 </sst>
 </file>
@@ -1935,7 +1938,9 @@
       <c r="A88" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B88" s="9"/>
+      <c r="B88" s="32" t="s">
+        <v>103</v>
+      </c>
       <c r="C88" s="9"/>
       <c r="D88" s="28"/>
     </row>

</xml_diff>